<commit_message>
Record verified nightly WhatsApp call attempt
</commit_message>
<xml_diff>
--- a/reports/amala-daily-report.xlsx
+++ b/reports/amala-daily-report.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calls" sheetId="1" r:id="Rf0b1ac78b40a4b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversation" sheetId="2" r:id="Ra217e0d852094713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calls" sheetId="1" r:id="R29084b6e5c5b435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversation" sheetId="2" r:id="R0c9da318148d4b7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,6 +416,32 @@
         <x:v>Call accepted; 4 speech clips transcribed; 4 spoken replies queued; 2,167 RTP packets and 2,167 decoded audio frames recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="d">
+        <x:v>2026-10-20T15:35:23.270Z</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>Amala</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Raj</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="d">
+        <x:v>2026-10-20T15:36:13.652Z</x:v>
+      </x:c>
+      <x:c r="F6" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str">
+        <x:v>Unanswered</x:v>
+      </x:c>
+      <x:c r="H6" s="14" t="str">
+        <x:v>No answer within 45 seconds. Report audio was not played. Measured CLI attempt elapsed time was 50.4 seconds, including setup and ringing; connected call duration was 0 minutes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -584,6 +610,27 @@
         <x:v>Tamil output retained exactly as logged; no correction applied.</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>Amala</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>No caller speech captured.</x:v>
+      </x:c>
+      <x:c r="E9" s="14"/>
+      <x:c r="F9" s="14" t="str">
+        <x:v>Not played</x:v>
+      </x:c>
+      <x:c r="G9" s="14" t="str">
+        <x:v>Scheduled report attempt at 21:05 local was unanswered. No transcript or spoken Amala reply was captured.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
Correct nightly call report with caller feedback
</commit_message>
<xml_diff>
--- a/reports/amala-daily-report.xlsx
+++ b/reports/amala-daily-report.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calls" sheetId="1" r:id="R29084b6e5c5b435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversation" sheetId="2" r:id="R0c9da318148d4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calls" sheetId="1" r:id="Rb3c6212c3576468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversation" sheetId="2" r:id="R488dc550d3d846e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,14 +432,12 @@
       <x:c r="E6" s="13" t="d">
         <x:v>2026-10-20T15:36:13.652Z</x:v>
       </x:c>
-      <x:c r="F6" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="F6" s="15"/>
       <x:c r="G6" s="14" t="str">
-        <x:v>Unanswered</x:v>
+        <x:v>Conflicting reports</x:v>
       </x:c>
       <x:c r="H6" s="14" t="str">
-        <x:v>No answer within 45 seconds. Report audio was not played. Measured CLI attempt elapsed time was 50.4 seconds, including setup and ringing; connected call duration was 0 minutes.</x:v>
+        <x:v>MeowCaller returned: recipient did not answer within 45 seconds; report audio was not played. Raj later reported that he answered and spoke, but Amala did not speak. Answer state and connected duration could not be independently verified. CLI elapsed time of 50.4 seconds includes setup and ringing.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -621,14 +619,16 @@
         <x:v>Amala</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>No caller speech captured.</x:v>
-      </x:c>
-      <x:c r="E9" s="14"/>
+        <x:v>Raj reports that he answered and spoke; his exact words were not captured.</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str">
+        <x:v>Raj reports that Amala did not speak.</x:v>
+      </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>Not played</x:v>
+        <x:v>No speech heard (caller report)</x:v>
       </x:c>
       <x:c r="G9" s="14" t="str">
-        <x:v>Scheduled report attempt at 21:05 local was unanswered. No transcript or spoken Amala reply was captured.</x:v>
+        <x:v>Caller report added after MeowCaller returned no answer. No call media or transcript is available to independently verify or quote exact speech.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>